<commit_message>
data: regenerate data due to typo
</commit_message>
<xml_diff>
--- a/data/t_pa.xlsx
+++ b/data/t_pa.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_MONASH_UNI\_Y3S1\FIT3179\DV2_repo\FIT3179_DV2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFCC03D5-A319-4D4F-B0D0-03F1B51C93B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A845D9B5-E87D-44C4-B057-B39081390E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$55</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="15">
   <si>
     <t>State Full Name</t>
   </si>
@@ -65,9 +68,6 @@
     <t>Queensland</t>
   </si>
   <si>
-    <t>Nothern Territory</t>
-  </si>
-  <si>
     <t>Australian Capital Territory</t>
   </si>
   <si>
@@ -79,6 +79,12 @@
   <si>
     <t>Percentage of Protected Area/Assigned area</t>
   </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>Northern Territory</t>
+  </si>
 </sst>
 </file>
 
@@ -87,7 +93,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="174" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -2915,29 +2921,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="174" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="174" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="174" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2346">
     <cellStyle name="20% - Accent1" xfId="17" builtinId="30" customBuiltin="1"/>
@@ -5563,7 +5567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
@@ -5571,9 +5575,10 @@
     <col min="3" max="3" width="27.109375" customWidth="1"/>
     <col min="4" max="4" width="19.44140625" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5581,18 +5586,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="3">
         <v>2014</v>
@@ -5607,7 +5615,7 @@
         <v>55.219140440343836</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -5624,7 +5632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
@@ -5641,9 +5649,9 @@
         <v>9.1032388101688362</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3">
         <v>2014</v>
@@ -5658,7 +5666,7 @@
         <v>18.644915251604129</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -5675,7 +5683,7 @@
         <v>8.156282906917145</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -5692,7 +5700,7 @@
         <v>29.865849533834549</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
@@ -5709,7 +5717,7 @@
         <v>44.088422106804941</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>2</v>
       </c>
@@ -5726,7 +5734,7 @@
         <v>17.632326346099152</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
@@ -5743,9 +5751,9 @@
         <v>21.517714545610279</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="3">
         <v>2016</v>
@@ -5759,8 +5767,12 @@
       <c r="E11" s="5">
         <v>55.480190189146391</v>
       </c>
+      <c r="H11">
+        <v>616</v>
+      </c>
+      <c r="I11" s="11"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
@@ -5776,8 +5788,12 @@
       <c r="E12" s="8">
         <v>0</v>
       </c>
+      <c r="H12">
+        <v>-2056</v>
+      </c>
+      <c r="I12" s="11"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>5</v>
       </c>
@@ -5793,10 +5809,14 @@
       <c r="E13" s="5">
         <v>9.2965766175545017</v>
       </c>
+      <c r="H13">
+        <v>154905</v>
+      </c>
+      <c r="I13" s="11"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B14" s="3">
         <v>2016</v>
@@ -5810,8 +5830,12 @@
       <c r="E14" s="5">
         <v>24.865979749299143</v>
       </c>
+      <c r="H14">
+        <v>8384674</v>
+      </c>
+      <c r="I14" s="11"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>8</v>
       </c>
@@ -5827,8 +5851,12 @@
       <c r="E15" s="5">
         <v>8.4414182757184939</v>
       </c>
+      <c r="H15">
+        <v>493209</v>
+      </c>
+      <c r="I15" s="11"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
@@ -5844,8 +5872,12 @@
       <c r="E16" s="5">
         <v>30.063239458149678</v>
       </c>
+      <c r="H16">
+        <v>194275</v>
+      </c>
+      <c r="I16" s="11"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>7</v>
       </c>
@@ -5861,8 +5893,12 @@
       <c r="E17" s="5">
         <v>42.313864490147971</v>
       </c>
+      <c r="H17">
+        <v>-121379</v>
+      </c>
+      <c r="I17" s="11"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>2</v>
       </c>
@@ -5878,8 +5914,12 @@
       <c r="E18" s="5">
         <v>17.220926607771762</v>
       </c>
+      <c r="H18">
+        <v>-95332</v>
+      </c>
+      <c r="I18" s="11"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -5895,10 +5935,14 @@
       <c r="E19" s="5">
         <v>23.259780859129556</v>
       </c>
+      <c r="H19">
+        <v>4402330</v>
+      </c>
+      <c r="I19" s="11"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20" s="3">
         <v>2018</v>
@@ -5912,8 +5956,12 @@
       <c r="E20" s="5">
         <v>55.654546669936678</v>
       </c>
+      <c r="H20">
+        <v>412</v>
+      </c>
+      <c r="I20" s="11"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>6</v>
       </c>
@@ -5923,14 +5971,18 @@
       <c r="C21" s="4">
         <v>40166.650496270013</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="6">
         <v>0</v>
       </c>
       <c r="E21" s="8">
         <v>0</v>
       </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>5</v>
       </c>
@@ -5946,10 +5998,14 @@
       <c r="E22" s="5">
         <v>9.3061861975110478</v>
       </c>
+      <c r="H22">
+        <v>7117</v>
+      </c>
+      <c r="I22" s="11"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B23" s="3">
         <v>2018</v>
@@ -5963,8 +6019,12 @@
       <c r="E23" s="5">
         <v>24.859532879905263</v>
       </c>
+      <c r="H23">
+        <v>-8589</v>
+      </c>
+      <c r="I23" s="11"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
@@ -5980,8 +6040,12 @@
       <c r="E24" s="5">
         <v>8.6802822669473105</v>
       </c>
+      <c r="H24">
+        <v>413219</v>
+      </c>
+      <c r="I24" s="11"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>4</v>
       </c>
@@ -5997,8 +6061,12 @@
       <c r="E25" s="5">
         <v>30.128877513100878</v>
       </c>
+      <c r="H25">
+        <v>67632</v>
+      </c>
+      <c r="I25" s="11"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>7</v>
       </c>
@@ -6014,8 +6082,12 @@
       <c r="E26" s="5">
         <v>42.350264019858528</v>
       </c>
+      <c r="H26">
+        <v>2490</v>
+      </c>
+      <c r="I26" s="11"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>2</v>
       </c>
@@ -6031,8 +6103,12 @@
       <c r="E27" s="5">
         <v>17.503957486354327</v>
       </c>
+      <c r="H27">
+        <v>64374</v>
+      </c>
+      <c r="I27" s="11"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
@@ -6048,10 +6124,14 @@
       <c r="E28" s="5">
         <v>23.387385250008432</v>
       </c>
+      <c r="H28">
+        <v>322458</v>
+      </c>
+      <c r="I28" s="11"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B29" s="3">
         <v>2020</v>
@@ -6065,8 +6145,12 @@
       <c r="E29" s="5">
         <v>55.857875823974609</v>
       </c>
+      <c r="H29">
+        <v>479</v>
+      </c>
+      <c r="I29" s="11"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>6</v>
       </c>
@@ -6076,14 +6160,18 @@
       <c r="C30" s="4">
         <v>40166.65086094274</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="9">
         <v>0</v>
       </c>
       <c r="E30" s="5">
         <v>0</v>
       </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30" s="11"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>5</v>
       </c>
@@ -6099,10 +6187,14 @@
       <c r="E31" s="5">
         <v>9.6069908142089844</v>
       </c>
+      <c r="H31">
+        <v>240990</v>
+      </c>
+      <c r="I31" s="11"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B32" s="3">
         <v>2020</v>
@@ -6116,8 +6208,12 @@
       <c r="E32" s="5">
         <v>24.859285354614261</v>
       </c>
+      <c r="H32">
+        <v>-334</v>
+      </c>
+      <c r="I32" s="11"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>8</v>
       </c>
@@ -6133,8 +6229,12 @@
       <c r="E33" s="5">
         <v>8.7124214172363281</v>
       </c>
+      <c r="H33">
+        <v>55592</v>
+      </c>
+      <c r="I33" s="11"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>4</v>
       </c>
@@ -6150,8 +6250,12 @@
       <c r="E34" s="5">
         <v>30.126926422119141</v>
       </c>
+      <c r="H34">
+        <v>-1921</v>
+      </c>
+      <c r="I34" s="11"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>7</v>
       </c>
@@ -6167,8 +6271,12 @@
       <c r="E35" s="5">
         <v>42.297988891601563</v>
       </c>
+      <c r="H35">
+        <v>-3576</v>
+      </c>
+      <c r="I35" s="11"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>2</v>
       </c>
@@ -6184,8 +6292,12 @@
       <c r="E36" s="5">
         <v>17.573024749755859</v>
       </c>
+      <c r="H36">
+        <v>15709</v>
+      </c>
+      <c r="I36" s="11"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>3</v>
       </c>
@@ -6201,10 +6313,14 @@
       <c r="E37" s="5">
         <v>23.303108215332031</v>
       </c>
+      <c r="H37">
+        <v>-212971</v>
+      </c>
+      <c r="I37" s="11"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B38" s="3">
         <v>2022</v>
@@ -6218,8 +6334,12 @@
       <c r="E38" s="5">
         <v>55.935256958007813</v>
       </c>
+      <c r="H38">
+        <v>182</v>
+      </c>
+      <c r="I38" s="11"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>6</v>
       </c>
@@ -6229,14 +6349,18 @@
       <c r="C39" s="4">
         <v>50312.781749716203</v>
       </c>
-      <c r="D39" s="10">
+      <c r="D39" s="9">
         <v>0</v>
       </c>
       <c r="E39" s="5">
         <v>0</v>
       </c>
+      <c r="H39">
+        <v>10146</v>
+      </c>
+      <c r="I39" s="11"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>5</v>
       </c>
@@ -6252,10 +6376,14 @@
       <c r="E40" s="5">
         <v>10.197736740112299</v>
       </c>
+      <c r="H40">
+        <v>473276</v>
+      </c>
+      <c r="I40" s="11"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B41" s="3">
         <v>2022</v>
@@ -6269,8 +6397,12 @@
       <c r="E41" s="5">
         <v>24.882425308227539</v>
       </c>
+      <c r="H41">
+        <v>31189</v>
+      </c>
+      <c r="I41" s="11"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>8</v>
       </c>
@@ -6286,8 +6418,12 @@
       <c r="E42" s="5">
         <v>8.8312854766845703</v>
       </c>
+      <c r="H42">
+        <v>205604</v>
+      </c>
+      <c r="I42" s="11"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>4</v>
       </c>
@@ -6303,8 +6439,12 @@
       <c r="E43" s="5">
         <v>30.195270538330082</v>
       </c>
+      <c r="H43">
+        <v>67273</v>
+      </c>
+      <c r="I43" s="11"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>7</v>
       </c>
@@ -6320,8 +6460,12 @@
       <c r="E44" s="5">
         <v>42.307548522949219</v>
       </c>
+      <c r="H44">
+        <v>654</v>
+      </c>
+      <c r="I44" s="11"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>2</v>
       </c>
@@ -6337,8 +6481,12 @@
       <c r="E45" s="5">
         <v>17.643430709838871</v>
       </c>
+      <c r="H45">
+        <v>16013</v>
+      </c>
+      <c r="I45" s="11"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>3</v>
       </c>
@@ -6354,42 +6502,54 @@
       <c r="E46" s="5">
         <v>30.13150787353516</v>
       </c>
+      <c r="H46">
+        <v>17255455</v>
+      </c>
+      <c r="I46" s="11"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B47" s="3">
         <v>2024</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="4">
         <v>131902</v>
       </c>
       <c r="D47" s="4">
         <v>235814.853081598</v>
       </c>
-      <c r="E47" s="12">
+      <c r="E47" s="10">
         <v>55.934715792538356</v>
       </c>
+      <c r="H47">
+        <v>-2</v>
+      </c>
+      <c r="I47" s="11"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B48" s="3">
         <v>2024</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48" s="4">
         <v>9681</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D48" s="9">
         <v>0</v>
       </c>
-      <c r="E48" s="12">
+      <c r="E48" s="10">
         <v>0</v>
       </c>
+      <c r="H48">
+        <v>-40632</v>
+      </c>
+      <c r="I48" s="11"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>5</v>
       </c>
@@ -6402,13 +6562,17 @@
       <c r="D49" s="4">
         <v>80115006.5110192</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="10">
         <v>10.441309542307987</v>
       </c>
+      <c r="H49">
+        <v>195138</v>
+      </c>
+      <c r="I49" s="11"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B50" s="3">
         <v>2024</v>
@@ -6419,11 +6583,15 @@
       <c r="D50" s="4">
         <v>134779162.69051</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="10">
         <v>24.639371053054575</v>
       </c>
+      <c r="H50">
+        <v>-327587</v>
+      </c>
+      <c r="I50" s="11"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -6436,11 +6604,15 @@
       <c r="D51" s="4">
         <v>172974215.256347</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="10">
         <v>9.3558179512458111</v>
       </c>
+      <c r="H51">
+        <v>907307</v>
+      </c>
+      <c r="I51" s="11"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>4</v>
       </c>
@@ -6453,11 +6625,15 @@
       <c r="D52" s="4">
         <v>98432191.357677802</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="10">
         <v>30.440771531811894</v>
       </c>
+      <c r="H52">
+        <v>241651</v>
+      </c>
+      <c r="I52" s="11"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>7</v>
       </c>
@@ -6470,11 +6646,15 @@
       <c r="D53" s="4">
         <v>6840139.3646279303</v>
       </c>
-      <c r="E53" s="12">
+      <c r="E53" s="10">
         <v>42.806946162674791</v>
       </c>
+      <c r="H53">
+        <v>34159</v>
+      </c>
+      <c r="I53" s="11"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>2</v>
       </c>
@@ -6487,11 +6667,15 @@
       <c r="D54" s="4">
         <v>22744373.104050402</v>
       </c>
-      <c r="E54" s="12">
+      <c r="E54" s="10">
         <v>17.690302579306515</v>
       </c>
+      <c r="H54">
+        <v>10661</v>
+      </c>
+      <c r="I54" s="11"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>3</v>
       </c>
@@ -6504,20 +6688,19 @@
       <c r="D55" s="4">
         <v>252701298.390847</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="10">
         <v>31.133286375035702</v>
       </c>
+      <c r="H55">
+        <v>2531509</v>
+      </c>
+      <c r="I55" s="11"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D56" s="4"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D57" s="13"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D58" s="13"/>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:E55" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>